<commit_message>
feat(basic): complete Basic course overhaul
- Fixed shopping list parser for lime/chili/grillad kyckling
- Updated all week 1-6 shopping lists with correct amounts
- Applied fuzzy matching for 383 recipe images
- Cleaned up invalid 'Energi: X kcal' recipe entries
- Updated all curated shopping list files with improved parser
- All Basic weeks now have correct recipes, nutrition, and shopping lists
</commit_message>
<xml_diff>
--- a/public/WEEK2_SHOPPING_LIST.xlsx
+++ b/public/WEEK2_SHOPPING_LIST.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Vecka 2 Inköpslista" sheetId="1" r:id="rId1"/>
+    <sheet name="Vecka 2" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -541,13 +541,10 @@
         <v>Frukt/Grönt</v>
       </c>
       <c r="C9" t="str">
-        <v>ul lök</v>
+        <v>gul lök</v>
       </c>
       <c r="D9">
         <v>0.5</v>
-      </c>
-      <c r="E9" t="str">
-        <v>g</v>
       </c>
     </row>
     <row r="10">
@@ -1333,13 +1330,10 @@
         <v>Kött/fisk/fågel/ägg/vego</v>
       </c>
       <c r="C60" t="str">
-        <v>rillad kyckling</v>
+        <v>grillad kyckling</v>
       </c>
       <c r="D60">
         <v>0.5</v>
-      </c>
-      <c r="E60" t="str">
-        <v>g</v>
       </c>
     </row>
     <row r="61">

</xml_diff>